<commit_message>
Add FNYSZ 30-day rule implementation and update test data for unpaid leave scenarios
</commit_message>
<xml_diff>
--- a/solutions/tools/tvSearch/jogszabalyok/test_input.xlsx
+++ b/solutions/tools/tvSearch/jogszabalyok/test_input.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -887,6 +887,32 @@
         <v>8</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1990.01.01</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1990.02.14</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>fizetés nélküli szabadság</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -898,7 +924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1328,6 +1354,34 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1990.01.01</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1990.02.14</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>45</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>fizetés nélküli szabadság</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>